<commit_message>
p2 | back 1.35
</commit_message>
<xml_diff>
--- a/optimization_results/top10_solutions.xlsx
+++ b/optimization_results/top10_solutions.xlsx
@@ -487,139 +487,139 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B2" t="n">
-        <v>90</v>
+        <v>136.5</v>
       </c>
       <c r="C2" t="n">
-        <v>0.303448275862069</v>
+        <v>0.3</v>
       </c>
       <c r="D2" t="n">
-        <v>0.7103448275862069</v>
+        <v>0.5</v>
       </c>
       <c r="E2" t="n">
-        <v>17827.10677765862</v>
+        <v>17840.72567161533</v>
       </c>
       <c r="F2" t="n">
-        <v>3.328293792306097</v>
+        <v>4.280440570810409</v>
       </c>
       <c r="G2" t="n">
         <v>1800</v>
       </c>
       <c r="H2" t="n">
-        <v>17890.56127990493</v>
+        <v>17908.60179097421</v>
       </c>
       <c r="I2" t="n">
-        <v>11.11952698793173</v>
+        <v>11.41450818882776</v>
       </c>
       <c r="J2" t="n">
-        <v>1797.527510107015</v>
+        <v>1798.775</v>
       </c>
       <c r="K2" t="n">
-        <v>4.640000000000001</v>
+        <v>4.65</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B3" t="n">
-        <v>130</v>
+        <v>140</v>
       </c>
       <c r="C3" t="n">
-        <v>0.303448275862069</v>
+        <v>0</v>
       </c>
       <c r="D3" t="n">
-        <v>0.5068965517241379</v>
+        <v>0.7000000000000001</v>
       </c>
       <c r="E3" t="n">
-        <v>17839.23217407936</v>
+        <v>17800</v>
       </c>
       <c r="F3" t="n">
-        <v>4.123467654420538</v>
+        <v>0</v>
       </c>
       <c r="G3" t="n">
         <v>1800</v>
       </c>
       <c r="H3" t="n">
-        <v>17904.76773759828</v>
+        <v>17897.26952286085</v>
       </c>
       <c r="I3" t="n">
-        <v>11.01153294078212</v>
+        <v>11.94319565370445</v>
       </c>
       <c r="J3" t="n">
-        <v>1798.740973840666</v>
+        <v>1797.599</v>
       </c>
       <c r="K3" t="n">
-        <v>4.640000000000001</v>
+        <v>4.65</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B4" t="n">
-        <v>130</v>
+        <v>119</v>
       </c>
       <c r="C4" t="n">
-        <v>0.5068965517241379</v>
+        <v>1.05</v>
       </c>
       <c r="D4" t="n">
-        <v>0.303448275862069</v>
+        <v>0</v>
       </c>
       <c r="E4" t="n">
-        <v>17865.53556351892</v>
+        <v>17924.47452752656</v>
       </c>
       <c r="F4" t="n">
-        <v>6.888065286361579</v>
+        <v>10.89011005631989</v>
       </c>
       <c r="G4" t="n">
         <v>1800</v>
       </c>
       <c r="H4" t="n">
-        <v>17904.76773759828</v>
+        <v>17924.47452752656</v>
       </c>
       <c r="I4" t="n">
-        <v>11.01153294078212</v>
+        <v>10.89011005631989</v>
       </c>
       <c r="J4" t="n">
-        <v>1799.548803804994</v>
+        <v>1800</v>
       </c>
       <c r="K4" t="n">
-        <v>4.640000000000001</v>
+        <v>4.649999999999999</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B5" t="n">
-        <v>90</v>
+        <v>98</v>
       </c>
       <c r="C5" t="n">
-        <v>0.9137931034482759</v>
+        <v>0.45</v>
       </c>
       <c r="D5" t="n">
-        <v>0.303448275862069</v>
+        <v>0.5</v>
       </c>
       <c r="E5" t="n">
-        <v>17881.92842603272</v>
+        <v>17843.85841558574</v>
       </c>
       <c r="F5" t="n">
-        <v>7.167808498384991</v>
+        <v>4.609705230103518</v>
       </c>
       <c r="G5" t="n">
         <v>1800</v>
       </c>
       <c r="H5" t="n">
-        <v>17909.13484675302</v>
+        <v>17892.58998845879</v>
       </c>
       <c r="I5" t="n">
-        <v>9.548061886527933</v>
+        <v>9.731599930218538</v>
       </c>
       <c r="J5" t="n">
-        <v>1799.548803804994</v>
+        <v>1798.775</v>
       </c>
       <c r="K5" t="n">
         <v>4.640000000000001</v>
@@ -627,212 +627,212 @@
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B6" t="n">
-        <v>110</v>
+        <v>133</v>
       </c>
       <c r="C6" t="n">
-        <v>0.9137931034482759</v>
+        <v>0.45</v>
       </c>
       <c r="D6" t="n">
-        <v>0.1</v>
+        <v>0.3</v>
       </c>
       <c r="E6" t="n">
-        <v>17900.13474292888</v>
+        <v>17859.52213543779</v>
       </c>
       <c r="F6" t="n">
-        <v>8.760654831359433</v>
+        <v>6.256028526569059</v>
       </c>
       <c r="G6" t="n">
         <v>1800</v>
       </c>
       <c r="H6" t="n">
-        <v>17911.09288460789</v>
+        <v>17899.20355906299</v>
       </c>
       <c r="I6" t="n">
-        <v>9.719368001583673</v>
+        <v>10.42671421094843</v>
       </c>
       <c r="J6" t="n">
-        <v>1799.951</v>
+        <v>1799.559</v>
       </c>
       <c r="K6" t="n">
-        <v>4.64</v>
+        <v>4.640000000000001</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B7" t="n">
-        <v>110</v>
+        <v>98</v>
       </c>
       <c r="C7" t="n">
-        <v>0.5068965517241379</v>
+        <v>1.05</v>
       </c>
       <c r="D7" t="n">
-        <v>0.5068965517241379</v>
+        <v>0.2</v>
       </c>
       <c r="E7" t="n">
-        <v>17855.4531691314</v>
+        <v>17902.50843443364</v>
       </c>
       <c r="F7" t="n">
-        <v>5.828362934613644</v>
+        <v>8.968325928734027</v>
       </c>
       <c r="G7" t="n">
         <v>1800</v>
       </c>
       <c r="H7" t="n">
-        <v>17910.90633826279</v>
+        <v>17922.03385051624</v>
       </c>
       <c r="I7" t="n">
-        <v>11.65672586922729</v>
+        <v>10.67657848658813</v>
       </c>
       <c r="J7" t="n">
-        <v>1798.740973840666</v>
+        <v>1799.804</v>
       </c>
       <c r="K7" t="n">
-        <v>4.64</v>
+        <v>4.640000000000001</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="B8" t="n">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="C8" t="n">
-        <v>0.1</v>
+        <v>0.8999999999999999</v>
       </c>
       <c r="D8" t="n">
-        <v>0.7103448275862069</v>
+        <v>0.2</v>
       </c>
       <c r="E8" t="n">
-        <v>17810.91800766805</v>
+        <v>17900.41642556765</v>
       </c>
       <c r="F8" t="n">
-        <v>1.340562777456622</v>
+        <v>8.785298868963944</v>
       </c>
       <c r="G8" t="n">
         <v>1800</v>
       </c>
       <c r="H8" t="n">
-        <v>17888.47351041354</v>
+        <v>17922.7311868049</v>
       </c>
       <c r="I8" t="n">
-        <v>10.86318112766573</v>
+        <v>10.73758750651149</v>
       </c>
       <c r="J8" t="n">
-        <v>1797.527510107015</v>
+        <v>1799.804</v>
       </c>
       <c r="K8" t="n">
-        <v>4.64</v>
+        <v>4.640000000000001</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B9" t="n">
-        <v>110</v>
+        <v>140</v>
       </c>
       <c r="C9" t="n">
-        <v>0.7103448275862069</v>
+        <v>0</v>
       </c>
       <c r="D9" t="n">
-        <v>0.303448275862069</v>
+        <v>0.6000000000000001</v>
       </c>
       <c r="E9" t="n">
-        <v>17877.70988327257</v>
+        <v>17800</v>
       </c>
       <c r="F9" t="n">
-        <v>8.167637853948371</v>
+        <v>0</v>
       </c>
       <c r="G9" t="n">
         <v>1800</v>
       </c>
       <c r="H9" t="n">
-        <v>17910.90633826279</v>
+        <v>17883.37387673787</v>
       </c>
       <c r="I9" t="n">
-        <v>11.65672586922729</v>
+        <v>10.23702484603239</v>
       </c>
       <c r="J9" t="n">
-        <v>1799.548803804994</v>
+        <v>1798.236</v>
       </c>
       <c r="K9" t="n">
-        <v>4.630000000000001</v>
+        <v>4.640000000000001</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B10" t="n">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="C10" t="n">
-        <v>0.7103448275862069</v>
+        <v>0.45</v>
       </c>
       <c r="D10" t="n">
-        <v>0.1</v>
+        <v>0.4</v>
       </c>
       <c r="E10" t="n">
-        <v>17891.99342763758</v>
+        <v>17859.52213543779</v>
       </c>
       <c r="F10" t="n">
-        <v>8.048382037180295</v>
+        <v>6.256028526569059</v>
       </c>
       <c r="G10" t="n">
         <v>1800</v>
       </c>
       <c r="H10" t="n">
-        <v>17904.94395871277</v>
+        <v>17912.43070027138</v>
       </c>
       <c r="I10" t="n">
-        <v>9.18140669289985</v>
+        <v>11.81694277240822</v>
       </c>
       <c r="J10" t="n">
-        <v>1799.951</v>
+        <v>1799.216</v>
       </c>
       <c r="K10" t="n">
-        <v>4.630000000000001</v>
+        <v>4.640000000000001</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="B11" t="n">
-        <v>90</v>
+        <v>84</v>
       </c>
       <c r="C11" t="n">
-        <v>0.1</v>
+        <v>0.45</v>
       </c>
       <c r="D11" t="n">
-        <v>0.7103448275862069</v>
+        <v>0.7000000000000001</v>
       </c>
       <c r="E11" t="n">
-        <v>17808.91241261867</v>
+        <v>17837.59292764492</v>
       </c>
       <c r="F11" t="n">
-        <v>1.252557908640589</v>
+        <v>3.951175911517301</v>
       </c>
       <c r="G11" t="n">
         <v>1800</v>
       </c>
       <c r="H11" t="n">
-        <v>17872.22127466857</v>
+        <v>17896.07081509257</v>
       </c>
       <c r="I11" t="n">
-        <v>10.15003822519098</v>
+        <v>10.09744955165533</v>
       </c>
       <c r="J11" t="n">
-        <v>1797.527510107015</v>
+        <v>1797.599</v>
       </c>
       <c r="K11" t="n">
-        <v>4.630000000000001</v>
+        <v>4.640000000000001</v>
       </c>
     </row>
   </sheetData>

</xml_diff>